<commit_message>
Changed Extended Date to Extended Expiry Date
</commit_message>
<xml_diff>
--- a/public/templates/TI_TE_Migration_Template.xlsx
+++ b/public/templates/TI_TE_Migration_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MohammedFarhan\Documents\Open POs Expediting\expediting_tool\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3CDD716-8B84-4696-ADD8-DF3CE46177A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3827FCC0-E153-4AB1-B038-5D4F386D014B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{C667FC59-5E10-41D4-940A-A1C6BB4F1A45}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="10800" xr2:uid="{C667FC59-5E10-41D4-940A-A1C6BB4F1A45}"/>
   </bookViews>
   <sheets>
     <sheet name="Ti-Te" sheetId="2" r:id="rId1"/>
@@ -59,9 +59,6 @@
     <t>Movement type</t>
   </si>
   <si>
-    <t xml:space="preserve">Extended date </t>
-  </si>
-  <si>
     <t xml:space="preserve">Comments </t>
   </si>
   <si>
@@ -96,6 +93,9 @@
   </si>
   <si>
     <t>Status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extended Expiry date </t>
   </si>
 </sst>
 </file>
@@ -974,7 +974,7 @@
     <tableColumn id="11" xr3:uid="{08425836-06DE-4477-A1D4-A9C5FF0B346D}" name="Movement type" dataDxfId="5"/>
     <tableColumn id="3" xr3:uid="{8CA8B099-3273-4407-88B2-53E27AE979B9}" name="Import Date " dataDxfId="4"/>
     <tableColumn id="4" xr3:uid="{E5184E22-3C57-4FB5-84D8-6D618E9EC437}" name="Expiry Date"/>
-    <tableColumn id="8" xr3:uid="{87E3B8DB-A377-411C-9E71-101769D4D70C}" name="Extended date " dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{87E3B8DB-A377-411C-9E71-101769D4D70C}" name="Extended Expiry date " dataDxfId="3"/>
     <tableColumn id="13" xr3:uid="{39A2AEC4-3ED6-4262-9E5E-AB22D526036E}" name="Deposit (USD)" dataDxfId="2"/>
     <tableColumn id="7" xr3:uid="{F98088D7-5C65-4547-8FAB-BCC11E03CBE0}" name="Comments " dataDxfId="1"/>
     <tableColumn id="19" xr3:uid="{CCC13C15-C3B1-4BDE-946C-FA5BB621BF8E}" name="Status" dataDxfId="0"/>
@@ -1315,7 +1315,7 @@
     <col min="11" max="11" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="29.140625" customWidth="1"/>
     <col min="13" max="14" width="19.140625" customWidth="1"/>
-    <col min="15" max="15" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="25.28515625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="25.42578125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="31" customWidth="1"/>
     <col min="18" max="18" width="23.28515625" customWidth="1"/>
@@ -1352,22 +1352,22 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>10</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>3</v>
@@ -1376,31 +1376,31 @@
         <v>4</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="L2" s="2" t="s">
         <v>5</v>
       </c>
       <c r="M2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="N2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="O2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="P2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="O2" s="3" t="s">
+      <c r="Q2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="P2" s="2" t="s">
+      <c r="R2" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="Q2" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="R2" s="2" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">

</xml_diff>